<commit_message>
Tech Stack Research added
</commit_message>
<xml_diff>
--- a/research/literature-survey/Literature_Analysis.xlsx
+++ b/research/literature-survey/Literature_Analysis.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FraudLens\research\literature-survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D27872E9-1EF1-46F9-998E-F07CCCC49AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB2D04B-02E1-41D0-AFB9-B559A170AD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{660EF063-B9AA-4630-87BF-F609F9B26BAB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{660EF063-B9AA-4630-87BF-F609F9B26BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="421">
   <si>
     <t>TECHNOLOGY COMPARISION</t>
   </si>
@@ -892,13 +894,421 @@
   </si>
   <si>
     <t>Priority</t>
+  </si>
+  <si>
+    <t>TECHNOLOGY APPLICABILITY</t>
+  </si>
+  <si>
+    <t>Literature Evidence</t>
+  </si>
+  <si>
+    <t>Investigation Relevance</t>
+  </si>
+  <si>
+    <t>Data / Infrastructure Requirements</t>
+  </si>
+  <si>
+    <t>Explainability / Evidence Support</t>
+  </si>
+  <si>
+    <t>Integration Potential</t>
+  </si>
+  <si>
+    <t>Implementation Feasibility</t>
+  </si>
+  <si>
+    <t>Key Limitations</t>
+  </si>
+  <si>
+    <t>Applicability to FraudLens</t>
+  </si>
+  <si>
+    <t>Selection Decision</t>
+  </si>
+  <si>
+    <t>Useful for explicit transaction conditions, known suspicious indicators, and investigator-defined rules.</t>
+  </si>
+  <si>
+    <t>Transaction data; domain rules; thresholds; risk indicators.</t>
+  </si>
+  <si>
+    <t>High; rules are transparent and can be directly inspected by investigators.</t>
+  </si>
+  <si>
+    <t>High; can complement ML, graph analysis, and investigation workflows.</t>
+  </si>
+  <si>
+    <t>High; relatively straightforward to implement and test.</t>
+  </si>
+  <si>
+    <t>Requires domain knowledge and predefined rules; may struggle with novel or evolving fraud patterns.</t>
+  </si>
+  <si>
+    <t>Supporting Technology</t>
+  </si>
+  <si>
+    <t>Strong relevance for transaction-level fraud-risk assessment and anomaly classification.</t>
+  </si>
+  <si>
+    <t>Historical labelled/unlabelled transaction data; engineered features; training/evaluation infrastructure.</t>
+  </si>
+  <si>
+    <t>Medium; depends on model and explanation method; risk score alone is insufficient evidence.</t>
+  </si>
+  <si>
+    <t>High; can provide analytical signals to graph, case, and investigation components.</t>
+  </si>
+  <si>
+    <t>High; mature libraries and evaluation methods are available.</t>
+  </si>
+  <si>
+    <t>Class imbalance, concept drift, dataset dependence, and limited labels can affect generalization.</t>
+  </si>
+  <si>
+    <t>Primary Candidate</t>
+  </si>
+  <si>
+    <t>Applicable to complex sequential, temporal, and graph patterns, but greater complexity is not always necessary.</t>
+  </si>
+  <si>
+    <t>Larger datasets; greater computational resources; specialized model training.</t>
+  </si>
+  <si>
+    <t>Low to Medium depending on architecture; complex models may require additional explainability methods.</t>
+  </si>
+  <si>
+    <t>Medium; integration can be more complex than conventional ML.</t>
+  </si>
+  <si>
+    <t>Medium; feasible but increases implementation and evaluation complexity.</t>
+  </si>
+  <si>
+    <t>Requires more data and computation; interpretability and generalization can be challenging.</t>
+  </si>
+  <si>
+    <t>Optional / Future</t>
+  </si>
+  <si>
+    <t>Highly relevant for identifying unusual transaction or entity behavior that can become investigation leads.</t>
+  </si>
+  <si>
+    <t>Historical behavior; transaction features; normal-behavior baselines; labelled data may not always be required.</t>
+  </si>
+  <si>
+    <t>Medium to High depending on method; anomalies still require contextual investigation.</t>
+  </si>
+  <si>
+    <t>High; anomaly signals can feed case analysis, graph analysis, and investigator review.</t>
+  </si>
+  <si>
+    <t>High; multiple supervised, semi-supervised, and unsupervised approaches are available.</t>
+  </si>
+  <si>
+    <t>Anomalous activity does not necessarily represent fraud; false positives and threshold selection remain challenges.</t>
+  </si>
+  <si>
+    <t>Highly relevant for transaction history, velocity, chronological behavior, and suspicious activity periods.</t>
+  </si>
+  <si>
+    <t>Timestamps; transaction histories; sequence construction; temporal features.</t>
+  </si>
+  <si>
+    <t>Medium to High; chronological transaction evidence is naturally inspectable.</t>
+  </si>
+  <si>
+    <t>High; can connect directly with transaction analytics and fund-flow analysis.</t>
+  </si>
+  <si>
+    <t>High for feature-based/sequence analysis; more complex deep models may require additional resources.</t>
+  </si>
+  <si>
+    <t>Long sequences and changing temporal behavior can increase complexity; temporal patterns alone do not prove fraud.</t>
+  </si>
+  <si>
+    <t>Highly relevant for relationships, multi-hop fund flows, intermediary accounts, and coordinated activity.</t>
+  </si>
+  <si>
+    <t>Entity and transaction relationships; graph database/processing; relationship metadata.</t>
+  </si>
+  <si>
+    <t>High when paths, relationships, and transactions can be shown to investigators.</t>
+  </si>
+  <si>
+    <t>High; can integrate accounts, people, companies, transactions, and documents.</t>
+  </si>
+  <si>
+    <t>Medium to High; graph modelling and traversal are feasible, while large-scale processing can be complex.</t>
+  </si>
+  <si>
+    <t>Highly connected networks can be computationally expensive and difficult to interpret without focused views.</t>
+  </si>
+  <si>
+    <t>Strong relevance for integrating heterogeneous investigation entities, relationships, concepts, and evidence.</t>
+  </si>
+  <si>
+    <t>Entity/relation extraction; graph schema; entity identifiers; provenance metadata.</t>
+  </si>
+  <si>
+    <t>High potential because relationships and provenance can be explicitly represented.</t>
+  </si>
+  <si>
+    <t>High; provides a common representation connecting documents, entities, transactions, and cases.</t>
+  </si>
+  <si>
+    <t>Medium; requires careful schema and extraction design.</t>
+  </si>
+  <si>
+    <t>Graph quality depends on accurate extraction, entity resolution, and relationship provenance.</t>
+  </si>
+  <si>
+    <t>Important for linking the same person, company, or account across different investigation sources.</t>
+  </si>
+  <si>
+    <t>Names, identifiers, account information, company attributes, document references, similarity features.</t>
+  </si>
+  <si>
+    <t>Medium to High when match confidence and source records are retained.</t>
+  </si>
+  <si>
+    <t>High; directly supports integration of transaction, document, and entity data.</t>
+  </si>
+  <si>
+    <t>Medium to High; established matching methods are available, but domain-specific validation is required.</t>
+  </si>
+  <si>
+    <t>False matches and missed matches can create incorrect or fragmented investigation relationships.</t>
+  </si>
+  <si>
+    <t>Essential where investigation documents are scanned, image-based, tabular, or visually structured.</t>
+  </si>
+  <si>
+    <t>Document files; OCR engine; layout information; extraction pipeline; validation mechanisms.</t>
+  </si>
+  <si>
+    <t>High when extracted fields retain document/page provenance and can be verified.</t>
+  </si>
+  <si>
+    <t>High; extracted entities and evidence can feed RAG and the investigation graph.</t>
+  </si>
+  <si>
+    <t>High for an initial prototype using established OCR/document-processing tools.</t>
+  </si>
+  <si>
+    <t>OCR and layout errors can propagate into extraction and retrieval; complex documents require validation.</t>
+  </si>
+  <si>
+    <t>Highly relevant for retrieving supporting evidence from investigation documents and answering document-grounded questions.</t>
+  </si>
+  <si>
+    <t>Document corpus; OCR/text extraction; embeddings or lexical index; metadata; retrieval/reranking infrastructure.</t>
+  </si>
+  <si>
+    <t>High if retrieved passages/pages and source metadata are exposed to the investigator.</t>
+  </si>
+  <si>
+    <t>High; naturally connects documents, cases, findings, and AI investigation assistance.</t>
+  </si>
+  <si>
+    <t>Medium to High; prototype implementation is feasible, but retrieval evaluation is required.</t>
+  </si>
+  <si>
+    <t>Incorrect retrieval can lead to incomplete or unsupported AI responses; OCR and chunking quality affect performance.</t>
+  </si>
+  <si>
+    <t>Highly relevant because investigation outputs need understandable analytical reasoning and supporting context.</t>
+  </si>
+  <si>
+    <t>Model explanations; graph paths; rules; feature contributions; evidence references.</t>
+  </si>
+  <si>
+    <t>Very High; directly supports investigator verification.</t>
+  </si>
+  <si>
+    <t>High; can operate across ML, graph, and evidence layers.</t>
+  </si>
+  <si>
+    <t>Medium to High; feasibility depends on selected analytical models.</t>
+  </si>
+  <si>
+    <t>Explanations can be incomplete or model-dependent and do not independently establish fraud.</t>
+  </si>
+  <si>
+    <t>Relevant to immediate transaction monitoring but less central to the broader evidence-based investigation workflow.</t>
+  </si>
+  <si>
+    <t>Streaming transaction feeds; low-latency processing; online model inference; monitoring infrastructure.</t>
+  </si>
+  <si>
+    <t>Medium; real-time risk indicators require later investigation and evidence verification.</t>
+  </si>
+  <si>
+    <t>Medium; can connect to transaction-risk analysis but adds infrastructure complexity.</t>
+  </si>
+  <si>
+    <t>Medium to Low for the current prototype scope.</t>
+  </si>
+  <si>
+    <t>Latency, concept drift, delayed labels, and infrastructure requirements increase complexity.</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Selection Status</t>
+  </si>
+  <si>
+    <t>Selected Role in FraudLens</t>
+  </si>
+  <si>
+    <t>Literature Basis</t>
+  </si>
+  <si>
+    <t>Research Gap Addressed</t>
+  </si>
+  <si>
+    <t>Why Applicable</t>
+  </si>
+  <si>
+    <t>Expected Output / Function</t>
+  </si>
+  <si>
+    <t>Technology Selection</t>
+  </si>
+  <si>
+    <t>Core / Selected</t>
+  </si>
+  <si>
+    <t>Transaction-level fraud-risk assessment and analytical scoring</t>
+  </si>
+  <si>
+    <t>Recurring limitations in fraud detection including class imbalance, changing behavior, limited labels, and dataset dependence</t>
+  </si>
+  <si>
+    <t>Provides a practical and well-established foundation for transaction-level analytical signals and can be evaluated using appropriate fraud-detection metrics</t>
+  </si>
+  <si>
+    <t>Fraud-risk score; classification output; analytical risk signal</t>
+  </si>
+  <si>
+    <t>Identify unusual transaction or entity behavior that may warrant investigation</t>
+  </si>
+  <si>
+    <t>Need to identify suspicious activity beyond only known labelled fraud patterns</t>
+  </si>
+  <si>
+    <t>Can complement supervised ML by identifying deviations from expected behavior and generating investigation leads</t>
+  </si>
+  <si>
+    <t>Anomaly score; suspicious activity indicator; behavioral deviation</t>
+  </si>
+  <si>
+    <t>Analyze transaction history, timing, frequency, velocity, and chronological patterns</t>
+  </si>
+  <si>
+    <t>Need for richer temporal and behavioral transaction analysis</t>
+  </si>
+  <si>
+    <t>Directly supports investigation of transaction sequences, rapid activity, temporal ordering, and changes in behavior</t>
+  </si>
+  <si>
+    <t>Temporal features; transaction sequences; suspicious activity periods</t>
+  </si>
+  <si>
+    <t>Model relationships between accounts, entities, transactions, and fund flows</t>
+  </si>
+  <si>
+    <t>Transaction-level analysis may miss multi-entity and network-level activity</t>
+  </si>
+  <si>
+    <t>Supports relationship analysis, multi-hop fund-flow tracing, intermediary identification, and network-based investigation</t>
+  </si>
+  <si>
+    <t>Transaction graph; relationship paths; fund-flow network</t>
+  </si>
+  <si>
+    <t>Provide a structured representation connecting investigation entities, transactions, documents, relationships, and knowledge</t>
+  </si>
+  <si>
+    <t>Need for integrated representation and reasoning across heterogeneous investigation information</t>
+  </si>
+  <si>
+    <t>Provides a common graph representation with explicit relationships and provenance that can connect multiple investigation data types</t>
+  </si>
+  <si>
+    <t>Entity/relation graph; investigation context; knowledge relationships</t>
+  </si>
+  <si>
+    <t>Link records referring to the same person, company, account, or other entity across data sources</t>
+  </si>
+  <si>
+    <t>P18; supported by P16, P19, P20, P22</t>
+  </si>
+  <si>
+    <t>Identity matching and heterogeneous data integration remain important challenges</t>
+  </si>
+  <si>
+    <t>Enables reliable connection of transaction records, documents, companies, accounts, and people while preserving match confidence</t>
+  </si>
+  <si>
+    <t>Resolved entity links; entity-match confidence</t>
+  </si>
+  <si>
+    <t>Convert scanned and visually structured investigation documents into usable information</t>
+  </si>
+  <si>
+    <t>Document extraction and OCR quality can affect downstream evidence analysis</t>
+  </si>
+  <si>
+    <t>Enables ingestion and structured extraction from scanned statements, reports, forms, and other investigation documents</t>
+  </si>
+  <si>
+    <t>Extracted text; fields; entities; document structure; page metadata</t>
+  </si>
+  <si>
+    <t>Retrieve relevant document evidence for investigator questions and AI-assisted analysis</t>
+  </si>
+  <si>
+    <t>Retrieval quality is a critical limitation for document-grounded AI</t>
+  </si>
+  <si>
+    <t>Supports evidence-grounded responses by retrieving relevant document content and preserving source context</t>
+  </si>
+  <si>
+    <t>Retrieved passages/pages; evidence references; grounded answers</t>
+  </si>
+  <si>
+    <t>Expose analytical signals, patterns, relationships, and evidence supporting investigation findings</t>
+  </si>
+  <si>
+    <t>Complex analytical outputs can be difficult for investigators to interpret</t>
+  </si>
+  <si>
+    <t>Supports human verification by connecting findings to understandable signals, graph paths, rules, and evidence</t>
+  </si>
+  <si>
+    <t>Explainable findings; supporting signals; reasoning context</t>
+  </si>
+  <si>
+    <t>Supporting</t>
+  </si>
+  <si>
+    <t>Apply explicit domain rules and investigator-defined indicators alongside analytical models</t>
+  </si>
+  <si>
+    <t>ML/anomaly methods may benefit from explicit domain knowledge and transparent conditions</t>
+  </si>
+  <si>
+    <t>Provides interpretable deterministic checks and a complementary signal without making rules the sole detection mechanism</t>
+  </si>
+  <si>
+    <t>Risk rules; rule matches; investigator-defined indicators</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -919,6 +1329,23 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -945,11 +1372,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -959,7 +1383,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1279,282 +1712,282 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.44140625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="19.88671875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="24.77734375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="27.6640625" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="25.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="1" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="1" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="1" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="1" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1571,302 +2004,302 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="31.21875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="37" style="3" customWidth="1"/>
-    <col min="5" max="5" width="29.21875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="28.33203125" style="3" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="3"/>
+    <col min="1" max="1" width="29.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="31.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37" style="2" customWidth="1"/>
+    <col min="5" max="5" width="29.21875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.33203125" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="1" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="1" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="1" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="1" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="1" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="1" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="1" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="1" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -1883,323 +2316,323 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18" style="5" customWidth="1"/>
-    <col min="2" max="2" width="25.77734375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="42.44140625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="28.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="27.33203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="34.5546875" style="5" customWidth="1"/>
-    <col min="7" max="7" width="27" style="5" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="18" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="27" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="1" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="88.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="88.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="1" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="1" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="82.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="1" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="1" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="102" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="1" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="1" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="106.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="1" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="1" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="99" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="1" t="s">
         <v>233</v>
       </c>
     </row>
@@ -2216,260 +2649,260 @@
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="29" style="5" customWidth="1"/>
-    <col min="3" max="3" width="32.5546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="37.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="32.33203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="28.109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="39.109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" style="5" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="19.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="37.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="39.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="5" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="5" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="1" t="s">
         <v>241</v>
       </c>
     </row>
@@ -2479,4 +2912,762 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D59E892-15A2-4A9A-95AF-3E4C2AF25DDC}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.44140625" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="41.6640625" customWidth="1"/>
+    <col min="4" max="4" width="47.44140625" customWidth="1"/>
+    <col min="5" max="5" width="53" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="7" max="7" width="38.77734375" customWidth="1"/>
+    <col min="8" max="8" width="37.21875" customWidth="1"/>
+    <col min="9" max="9" width="43.77734375" customWidth="1"/>
+    <col min="10" max="10" width="31.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="25.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11" ht="18" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="K14" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4C3BE9C-B19A-41D5-A29B-E256753C6028}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="43.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="27.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="36.6640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="25.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>